<commit_message>
winter with 3 rainy days
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -8,9 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0130E74-85F0-4260-B64B-3C188B9B9DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B329515E-084A-4E54-8B8C-54C1BB6A2CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{85126765-781C-418F-98CB-143316E98FFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -71,7 +72,7 @@
     <author>tc={2CD69954-9FBF-4F0C-A085-7745F169BA9F}</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{4E18937C-0B14-4E86-B599-4BF7BA80B225}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{4E18937C-0B14-4E86-B599-4BF7BA80B225}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +80,7 @@
     This is fine for winter, but for the summer, this would highly bias the results towards the weekend.</t>
       </text>
     </comment>
-    <comment ref="A4" authorId="1" shapeId="0" xr:uid="{2CD69954-9FBF-4F0C-A085-7745F169BA9F}">
+    <comment ref="B4" authorId="1" shapeId="0" xr:uid="{2CD69954-9FBF-4F0C-A085-7745F169BA9F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -92,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
   <si>
     <t>Annual AF</t>
   </si>
@@ -161,18 +162,6 @@
   </si>
   <si>
     <t>Rainy Days</t>
-  </si>
-  <si>
-    <t>Sum</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Running Total</t>
-  </si>
-  <si>
-    <t>Count</t>
   </si>
   <si>
     <t>AF/year to m3/week</t>
@@ -182,7 +171,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,18 +186,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -237,20 +214,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -268,9 +247,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -292,8 +268,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:P6" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:P6" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:P9" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:P9" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{FADC07E8-CEDF-4B75-BBE4-A01ACB71EDD0}" name="Season"/>
     <tableColumn id="2" xr3:uid="{19D40EF6-9320-45FB-A774-40B56854F6B1}" name="Rainy Days"/>
@@ -310,7 +286,7 @@
     <tableColumn id="13" xr3:uid="{2AE3D243-D71B-48B9-87D2-BFD00350BF9A}" name="Total Replacement Cost ($)"/>
     <tableColumn id="14" xr3:uid="{B5251DEF-3E31-4ABB-B44C-AE5BAB4EED3A}" name="Degree of Flexibility"/>
     <tableColumn id="15" xr3:uid="{2C164AA9-7F5B-49E1-A3E8-CC250E8A10E0}" name="Levelized Cost of Water ($/m3)"/>
-    <tableColumn id="16" xr3:uid="{DD6FED5F-B3AC-4690-ADB6-A1351F19574D}" name="Total OPEX Cost" dataDxfId="1">
+    <tableColumn id="16" xr3:uid="{DD6FED5F-B3AC-4690-ADB6-A1351F19574D}" name="Total OPEX Cost" dataDxfId="0">
       <calculatedColumnFormula>M2+L2+K2+J2+I2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -592,10 +568,10 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="D1" dT="2026-08-21T19:08:40.15" personId="{D208FEB8-F7DA-4D83-AAE5-2EEFF5739FC7}" id="{4E18937C-0B14-4E86-B599-4BF7BA80B225}">
+  <threadedComment ref="E1" dT="2026-08-21T19:08:40.15" personId="{D208FEB8-F7DA-4D83-AAE5-2EEFF5739FC7}" id="{4E18937C-0B14-4E86-B599-4BF7BA80B225}">
     <text>This is fine for winter, but for the summer, this would highly bias the results towards the weekend.</text>
   </threadedComment>
-  <threadedComment ref="A4" dT="2026-08-21T19:09:12.49" personId="{D208FEB8-F7DA-4D83-AAE5-2EEFF5739FC7}" id="{2CD69954-9FBF-4F0C-A085-7745F169BA9F}">
+  <threadedComment ref="B4" dT="2026-08-21T19:09:12.49" personId="{D208FEB8-F7DA-4D83-AAE5-2EEFF5739FC7}" id="{2CD69954-9FBF-4F0C-A085-7745F169BA9F}">
     <text>Two Trains on for one day</text>
   </threadedComment>
 </ThreadedComments>
@@ -615,11 +591,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D2">
@@ -644,64 +620,63 @@
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <f>C4/$G$10</f>
         <v>1190.7306933411717</v>
       </c>
       <c r="C4">
         <v>28000</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <f>C5/$G$10</f>
         <v>1798.4286079070769</v>
       </c>
       <c r="C5">
         <v>42290</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <f>C6/$G$10</f>
         <v>2397.9615120043568</v>
       </c>
       <c r="C6">
         <v>56388</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="5"/>
+      <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="D7" s="1"/>
+      <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="D8" s="1"/>
+      <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="D9" s="1"/>
+      <c r="F9" s="1"/>
       <c r="G9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>8000</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>188119.78330000001</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>80541.55863</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="1"/>
       <c r="G10">
         <f>C10/B10</f>
         <v>23.514972912500003</v>
@@ -711,86 +686,86 @@
       <c r="B11">
         <v>9000</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="F11" s="2"/>
+      <c r="D11" s="3"/>
+      <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="4">
+      <c r="B12" s="3">
         <f>C12/$G$10</f>
         <v>9591.8460480174272</v>
       </c>
       <c r="C12">
         <v>225552</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>10000</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>11000</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>258664.69889999999</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>108042.46335199999</v>
       </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>12000</v>
       </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>13000</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B17">
         <v>14000</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>329209.6164</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>136028.56817899999</v>
       </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>15000</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>16000</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -803,11 +778,11 @@
       <c r="C20">
         <v>394716</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>171053.54809522501</v>
       </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -820,160 +795,218 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E02D5E1-F801-4839-8C05-CA5C31CB2DFA}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="B1:H22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" customWidth="1"/>
+    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.453125" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" customWidth="1"/>
+    <col min="7" max="7" width="10.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D1" s="1" t="s">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D2">
-        <v>0</v>
-      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
         <v>3</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>28000</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1191</v>
+      </c>
+      <c r="D4" s="3">
+        <v>28006.332369864798</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="3">
+        <v>16720.240035535448</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C5">
-        <v>42290</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1798</v>
+      </c>
+      <c r="D5" s="3">
+        <v>42292.226399718798</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="3">
+        <v>22368.52857086459</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C6">
-        <v>56388</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B10">
+        <v>2398</v>
+      </c>
+      <c r="D6" s="3">
+        <v>56388.904300408598</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="3">
+        <v>28772.571914996501</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C7">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C8">
+        <v>4000</v>
+      </c>
+      <c r="E8" s="1"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C9">
+        <v>5000</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C10">
+        <v>6000</v>
+      </c>
+      <c r="E10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C11">
+        <v>7000</v>
+      </c>
+      <c r="E11" s="1"/>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C12">
         <v>8000</v>
       </c>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B11">
+      <c r="D12" s="3">
+        <v>188119.78330000001</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12">
+        <f>D12/C12</f>
+        <v>23.514972912500003</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C13">
         <v>9000</v>
       </c>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B12">
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C14" s="3">
+        <f>D14/H12</f>
+        <v>9591.8460480174272</v>
+      </c>
+      <c r="D14">
+        <v>225552</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C15">
         <v>10000</v>
       </c>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B13">
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="C16">
         <v>11000</v>
       </c>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C14">
-        <v>225552</v>
-      </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B15">
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C17">
         <v>12000</v>
       </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B16">
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C18">
         <v>13000</v>
       </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B17">
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C19">
         <v>14000</v>
       </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B18">
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C20">
         <v>15000</v>
       </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B19">
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C21">
         <v>16000</v>
       </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
         <v>3</v>
       </c>
-      <c r="C20">
+      <c r="D22">
         <v>394716</v>
       </c>
-      <c r="D20" s="4">
+      <c r="E22" s="3">
         <v>158104.1957609462</v>
       </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="E1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -1000,56 +1033,56 @@
     <col min="13" max="13" width="25.36328125" customWidth="1"/>
     <col min="14" max="14" width="19.1796875" customWidth="1"/>
     <col min="15" max="15" width="28.6328125" customWidth="1"/>
-    <col min="16" max="16" width="16.26953125" style="4" customWidth="1"/>
+    <col min="16" max="16" width="16.26953125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1099,7 +1132,7 @@
       <c r="O2">
         <v>0.70492795036996803</v>
       </c>
-      <c r="P2" s="4">
+      <c r="P2" s="3">
         <f>M2+L2+K2+J2+I2</f>
         <v>158104.1957609462</v>
       </c>
@@ -1150,7 +1183,7 @@
       <c r="O3">
         <v>0.73773470848030298</v>
       </c>
-      <c r="P3" s="4">
+      <c r="P3" s="3">
         <f t="shared" ref="P3:P12" si="0">M3+L3+K3+J3+I3</f>
         <v>171053.54809522501</v>
       </c>
@@ -1201,7 +1234,7 @@
       <c r="O4">
         <v>1.0667868110000001</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="3">
         <f t="shared" si="0"/>
         <v>80541.55863</v>
       </c>
@@ -1252,7 +1285,7 @@
       <c r="O5">
         <v>0.88211430199999996</v>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="3">
         <f t="shared" si="0"/>
         <v>108042.46335199999</v>
       </c>
@@ -1303,43 +1336,178 @@
       <c r="O6">
         <v>0.77806027200000005</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="3">
         <f t="shared" si="0"/>
         <v>136028.56817899999</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P7" s="4">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>2398</v>
+      </c>
+      <c r="D7">
+        <v>10</v>
+      </c>
+      <c r="E7">
+        <v>56388.904300408598</v>
+      </c>
+      <c r="F7">
+        <v>148904.51312256299</v>
+      </c>
+      <c r="G7">
+        <v>3492.0724412416398</v>
+      </c>
+      <c r="H7">
+        <v>5287.8238927682696</v>
+      </c>
+      <c r="I7">
+        <v>10272.519814514601</v>
+      </c>
+      <c r="J7">
+        <v>4291.8348189990802</v>
+      </c>
+      <c r="K7">
+        <v>4008.2796281577898</v>
+      </c>
+      <c r="L7">
+        <v>8779.8963340099108</v>
+      </c>
+      <c r="M7">
+        <v>1420.0413193151201</v>
+      </c>
+      <c r="N7">
+        <v>7.1856287425149698E-2</v>
+      </c>
+      <c r="O7">
+        <v>2.6406704469603199</v>
+      </c>
+      <c r="P7" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>28772.571914996501</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P8" s="4">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>1798</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8">
+        <v>42292.226399718798</v>
+      </c>
+      <c r="F8">
+        <v>142505.590119726</v>
+      </c>
+      <c r="G8">
+        <v>2685.6739628165201</v>
+      </c>
+      <c r="H8">
+        <v>4056.7859256987999</v>
+      </c>
+      <c r="I8">
+        <v>7708.7043999531998</v>
+      </c>
+      <c r="J8">
+        <v>3463.15238966165</v>
+      </c>
+      <c r="K8">
+        <v>3039.2909147149098</v>
+      </c>
+      <c r="L8">
+        <v>6742.45988851532</v>
+      </c>
+      <c r="M8">
+        <v>1414.9209780195099</v>
+      </c>
+      <c r="N8">
+        <v>3.59281437125748E-2</v>
+      </c>
+      <c r="O8">
+        <v>3.36954571208561</v>
+      </c>
+      <c r="P8" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>22368.52857086459</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P9" s="4">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>1191</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>28006.332369864798</v>
+      </c>
+      <c r="F9">
+        <v>136852.18124310201</v>
+      </c>
+      <c r="G9">
+        <v>1795.6766797196899</v>
+      </c>
+      <c r="H9">
+        <v>2651.1746633135699</v>
+      </c>
+      <c r="I9">
+        <v>5102.7220616439199</v>
+      </c>
+      <c r="J9">
+        <v>3562.36888913341</v>
+      </c>
+      <c r="K9">
+        <v>2188.25642240973</v>
+      </c>
+      <c r="L9">
+        <v>4446.8513430332696</v>
+      </c>
+      <c r="M9">
+        <v>1420.0413193151201</v>
+      </c>
+      <c r="N9">
+        <v>7.1856287425149698E-2</v>
+      </c>
+      <c r="O9">
+        <v>4.8864727960722396</v>
+      </c>
+      <c r="P9" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>16720.240035535448</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P10" s="4">
+      <c r="P10" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P11" s="4">
+      <c r="P11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P12" s="4">
+      <c r="P12" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
0 rainy days, summer and winter sweep
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -8,9 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6AE8B90-1AC7-4C73-BBD6-11DE1BC07C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47938CA3-3BBE-45BA-89AD-A631B6094558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-94" yWindow="-94" windowWidth="33103" windowHeight="17983" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -213,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -221,7 +222,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -269,7 +269,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:P16" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:P16" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}"/>
+  <autoFilter ref="A1:P16" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Summer"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{FADC07E8-CEDF-4B75-BBE4-A01ACB71EDD0}" name="Season"/>
     <tableColumn id="2" xr3:uid="{19D40EF6-9320-45FB-A774-40B56854F6B1}" name="Rainy Days"/>
@@ -580,24 +586,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B1DDFCB-CD48-4284-8222-18B5894FE623}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" customWidth="1"/>
+    <col min="2" max="2" width="9.23046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.4609375" customWidth="1"/>
+    <col min="4" max="4" width="9.84375" customWidth="1"/>
+    <col min="5" max="5" width="9.4609375" customWidth="1"/>
+    <col min="6" max="6" width="10.3828125" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D2">
         <v>0</v>
       </c>
@@ -608,7 +614,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -616,7 +622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -630,7 +636,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B5" s="3">
         <f>C5/$G$10</f>
         <v>1798.4286079070769</v>
@@ -641,7 +647,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B6" s="3">
         <f>C6/$G$10</f>
         <v>2397.9615120043568</v>
@@ -651,22 +657,22 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D8" s="1"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B10">
         <v>8000</v>
       </c>
@@ -682,14 +688,19 @@
         <v>23.514972912500003</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B11">
         <v>9000</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="C11" s="3">
+        <v>211634.775495949</v>
+      </c>
+      <c r="D11" s="3">
+        <v>90145.456985227414</v>
+      </c>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B12" s="3">
         <f>C12/$G$10</f>
         <v>9591.8460480174272</v>
@@ -698,10 +709,9 @@
         <v>225552</v>
       </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="5"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B13">
         <v>10000</v>
       </c>
@@ -709,7 +719,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B14">
         <v>11000</v>
       </c>
@@ -722,7 +732,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B15">
         <v>12000</v>
       </c>
@@ -730,7 +740,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B16">
         <v>13000</v>
       </c>
@@ -738,7 +748,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B17">
         <v>14000</v>
       </c>
@@ -751,7 +761,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B18">
         <v>15000</v>
       </c>
@@ -759,7 +769,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B19">
         <v>16000</v>
       </c>
@@ -767,7 +777,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -784,7 +794,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="C21">
         <f>C20*4/7</f>
         <v>225552</v>
@@ -802,23 +812,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E02D5E1-F801-4839-8C05-CA5C31CB2DFA}">
   <dimension ref="B1:H22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.453125" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" customWidth="1"/>
-    <col min="7" max="7" width="10.36328125" customWidth="1"/>
+    <col min="3" max="3" width="9.23046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.4609375" customWidth="1"/>
+    <col min="5" max="5" width="9.84375" customWidth="1"/>
+    <col min="6" max="6" width="9.4609375" customWidth="1"/>
+    <col min="7" max="7" width="10.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.4">
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
       <c r="E2">
         <v>0</v>
       </c>
@@ -829,7 +839,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C3" t="s">
         <v>0</v>
       </c>
@@ -837,7 +847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -853,7 +863,7 @@
         <v>16720.240035535448</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C5">
         <v>1798</v>
       </c>
@@ -866,7 +876,7 @@
         <v>22368.52857086459</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C6">
         <v>2398</v>
       </c>
@@ -879,7 +889,7 @@
         <v>28772.571914996501</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C7">
         <v>3000</v>
       </c>
@@ -888,21 +898,21 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C8">
         <v>4000</v>
       </c>
       <c r="E8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C9">
         <v>5000</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C10">
         <v>6000</v>
       </c>
@@ -912,14 +922,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C11">
         <v>7000</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C12">
         <v>8000</v>
       </c>
@@ -932,13 +942,13 @@
         <v>23.514972912500003</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C13">
         <v>9000</v>
       </c>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C14" s="3">
         <f>D14/H12</f>
         <v>9591.8460480174272</v>
@@ -948,56 +958,56 @@
       </c>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C15">
         <v>10000</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C16">
         <v>11000</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C17">
         <v>12000</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C18">
         <v>13000</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C19">
         <v>14000</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C20">
         <v>15000</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C21">
         <v>16000</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.4">
       <c r="B22" t="s">
         <v>3</v>
       </c>
@@ -1022,27 +1032,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44889D92-5C1B-43B6-BE00-3D23C35CC93C}">
   <dimension ref="A1:P16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" customWidth="1"/>
-    <col min="3" max="3" width="22.26953125" customWidth="1"/>
-    <col min="4" max="4" width="28.81640625" customWidth="1"/>
-    <col min="5" max="5" width="26.90625" customWidth="1"/>
+    <col min="1" max="1" width="8.69140625" customWidth="1"/>
+    <col min="2" max="2" width="11.84375" customWidth="1"/>
+    <col min="3" max="3" width="22.23046875" customWidth="1"/>
+    <col min="4" max="4" width="28.84375" customWidth="1"/>
+    <col min="5" max="5" width="26.921875" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="20.08984375" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" customWidth="1"/>
-    <col min="9" max="9" width="18.453125" customWidth="1"/>
-    <col min="10" max="10" width="18.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.07421875" customWidth="1"/>
+    <col min="8" max="8" width="21.53515625" customWidth="1"/>
+    <col min="9" max="9" width="18.4609375" customWidth="1"/>
+    <col min="10" max="10" width="18.84375" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="22.54296875" customWidth="1"/>
-    <col min="13" max="13" width="25.36328125" customWidth="1"/>
-    <col min="14" max="14" width="19.1796875" customWidth="1"/>
-    <col min="15" max="15" width="28.6328125" customWidth="1"/>
-    <col min="16" max="16" width="16.26953125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="22.53515625" customWidth="1"/>
+    <col min="13" max="13" width="25.3828125" customWidth="1"/>
+    <col min="14" max="14" width="19.15234375" customWidth="1"/>
+    <col min="15" max="15" width="28.61328125" customWidth="1"/>
+    <col min="16" max="16" width="16.23046875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -1092,7 +1102,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1143,7 +1153,7 @@
         <v>158104.1957609462</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1194,7 +1204,7 @@
         <v>171053.54809522501</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1245,7 +1255,7 @@
         <v>80541.55863</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1296,7 +1306,7 @@
         <v>108042.46335199999</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1347,7 +1357,7 @@
         <v>136028.56817899999</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1398,7 +1408,7 @@
         <v>28772.571914996501</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1449,7 +1459,7 @@
         <v>22368.52857086459</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1500,7 +1510,7 @@
         <v>16720.240035535448</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1551,7 +1561,7 @@
         <v>90145.456985227414</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1602,7 +1612,7 @@
         <v>90891.797768890829</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1653,7 +1663,7 @@
         <v>41752.231305558547</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1704,7 +1714,7 @@
         <v>51495.778789739757</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1755,7 +1765,7 @@
         <v>60724.979693855727</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1806,7 +1816,7 @@
         <v>70388.430895292957</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Water target sweep for baseline costs summer
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -8,10 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{957FE4D1-DB70-47AD-A099-FAC1C4C9941E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14E49BC-EB75-4A27-B469-C3E5636FE192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -93,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="26">
   <si>
     <t>Annual AF</t>
   </si>
@@ -167,7 +166,10 @@
     <t>AF/year to m3/week</t>
   </si>
   <si>
-    <t>Column1</t>
+    <t>Flexible?</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -228,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -238,7 +240,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -290,11 +291,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:Q24" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:Q24" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Winter"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="1">
       <filters>
         <filter val="0"/>
@@ -323,7 +319,7 @@
     <tableColumn id="13" xr3:uid="{2AE3D243-D71B-48B9-87D2-BFD00350BF9A}" name="Total Replacement Cost ($)"/>
     <tableColumn id="14" xr3:uid="{B5251DEF-3E31-4ABB-B44C-AE5BAB4EED3A}" name="Degree of Flexibility"/>
     <tableColumn id="15" xr3:uid="{2C164AA9-7F5B-49E1-A3E8-CC250E8A10E0}" name="Levelized Cost of Water ($/m3)"/>
-    <tableColumn id="16" xr3:uid="{DD6FED5F-B3AC-4690-ADB6-A1351F19574D}" name="Column1" dataDxfId="0"/>
+    <tableColumn id="16" xr3:uid="{DD6FED5F-B3AC-4690-ADB6-A1351F19574D}" name="Flexible?" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -744,7 +740,7 @@
       <c r="B13">
         <v>10000</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="4">
         <v>235149.72602739499</v>
       </c>
       <c r="D13" s="3">
@@ -1213,7 +1209,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="3">
-        <f>N2+M2+L2+K2+J2</f>
+        <f t="shared" ref="C2:C24" si="0">N2+M2+L2+K2+J2</f>
         <v>158104.1957609462</v>
       </c>
       <c r="D2">
@@ -1255,8 +1251,11 @@
       <c r="P2">
         <v>0.70492795036996803</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q2" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1264,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3">
-        <f>N3+M3+L3+K3+J3</f>
+        <f t="shared" si="0"/>
         <v>171053.54809522501</v>
       </c>
       <c r="D3">
@@ -1306,8 +1305,11 @@
       <c r="P3">
         <v>0.73773470848030298</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q3" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1315,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="3">
-        <f>N4+M4+L4+K4+J4</f>
+        <f t="shared" si="0"/>
         <v>80541.55863</v>
       </c>
       <c r="D4">
@@ -1357,8 +1359,11 @@
       <c r="P4">
         <v>1.0667868110000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q4" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1366,7 +1371,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="3">
-        <f>N5+M5+L5+K5+J5</f>
+        <f t="shared" si="0"/>
         <v>90145.456985227414</v>
       </c>
       <c r="D5">
@@ -1408,8 +1413,11 @@
       <c r="P5">
         <v>0.99348767375321601</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q5" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1417,7 +1425,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="3">
-        <f>N6+M6+L6+K6+J6</f>
+        <f t="shared" si="0"/>
         <v>99135.784106883366</v>
       </c>
       <c r="D6">
@@ -1458,6 +1466,9 @@
       </c>
       <c r="P6">
         <v>0.93243811712477798</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
@@ -1468,7 +1479,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3">
-        <f>N7+M7+L7+K7+J7</f>
+        <f t="shared" si="0"/>
         <v>28772.571914996501</v>
       </c>
       <c r="D7">
@@ -1519,7 +1530,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="3">
-        <f>N8+M8+L8+K8+J8</f>
+        <f t="shared" si="0"/>
         <v>22368.52857086459</v>
       </c>
       <c r="D8">
@@ -1570,7 +1581,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="3">
-        <f>N9+M9+L9+K9+J9</f>
+        <f t="shared" si="0"/>
         <v>16720.240035535448</v>
       </c>
       <c r="D9">
@@ -1613,7 +1624,7 @@
         <v>4.8864727960722396</v>
       </c>
     </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1621,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="3">
-        <f>N10+M10+L10+K10+J10</f>
+        <f t="shared" si="0"/>
         <v>108042.46335199999</v>
       </c>
       <c r="D10">
@@ -1662,6 +1673,9 @@
       </c>
       <c r="P10">
         <v>0.88211430199999996</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
@@ -1672,7 +1686,7 @@
         <v>3</v>
       </c>
       <c r="C11" s="3">
-        <f>N11+M11+L11+K11+J11</f>
+        <f t="shared" si="0"/>
         <v>41752.231305558547</v>
       </c>
       <c r="D11">
@@ -1723,7 +1737,7 @@
         <v>3</v>
       </c>
       <c r="C12" s="3">
-        <f>N12+M12+L12+K12+J12</f>
+        <f t="shared" si="0"/>
         <v>51495.778789739757</v>
       </c>
       <c r="D12">
@@ -1774,7 +1788,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="3">
-        <f>N13+M13+L13+K13+J13</f>
+        <f t="shared" si="0"/>
         <v>60724.979693855727</v>
       </c>
       <c r="D13">
@@ -1825,7 +1839,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="3">
-        <f>N14+M14+L14+K14+J14</f>
+        <f t="shared" si="0"/>
         <v>70388.430895292957</v>
       </c>
       <c r="D14">
@@ -1876,7 +1890,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="3">
-        <f>N15+M15+L15+K15+J15</f>
+        <f t="shared" si="0"/>
         <v>80116.314065181752</v>
       </c>
       <c r="D15">
@@ -1927,7 +1941,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="3">
-        <f>N16+M16+L16+K16+J16</f>
+        <f t="shared" si="0"/>
         <v>90891.797768890829</v>
       </c>
       <c r="D16">
@@ -1970,7 +1984,7 @@
         <v>0.99711288227329198</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1978,7 +1992,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="3">
-        <f>N17+M17+L17+K17+J17</f>
+        <f t="shared" si="0"/>
         <v>117856.65704778227</v>
       </c>
       <c r="D17">
@@ -2020,8 +2034,11 @@
       <c r="P17">
         <v>0.84334790223742195</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q17" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2029,7 +2046,7 @@
         <v>0</v>
       </c>
       <c r="C18" s="3">
-        <f>N18+M18+L18+K18+J18</f>
+        <f t="shared" si="0"/>
         <v>126980.73146875472</v>
       </c>
       <c r="D18">
@@ -2071,8 +2088,11 @@
       <c r="P18">
         <v>0.80833055138049104</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q18" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2080,7 +2100,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="3">
-        <f>N19+M19+L19+K19+J19</f>
+        <f t="shared" si="0"/>
         <v>135947.17095224367</v>
       </c>
       <c r="D19">
@@ -2122,8 +2142,11 @@
       <c r="P19">
         <v>0.77781898176327602</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="Q19" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2131,7 +2154,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="3">
-        <f>N20+M20+L20+K20+J20</f>
+        <f t="shared" si="0"/>
         <v>75506.612155252791</v>
       </c>
       <c r="D20">
@@ -2173,8 +2196,11 @@
       <c r="P20">
         <v>1.0400222475155101</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="Q20" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2182,7 +2208,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="3">
-        <f>N21+M21+L21+K21+J21</f>
+        <f t="shared" si="0"/>
         <v>85155.50909649636</v>
       </c>
       <c r="D21">
@@ -2224,8 +2250,11 @@
       <c r="P21">
         <v>0.96998384928330195</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q21" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2233,7 +2262,7 @@
         <v>0</v>
       </c>
       <c r="C22" s="3">
-        <f>N22+M22+L22+K22+J22</f>
+        <f t="shared" si="0"/>
         <v>146231.12922675692</v>
       </c>
       <c r="D22">
@@ -2275,8 +2304,11 @@
       <c r="P22">
         <v>0.75491855067547597</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.4">
+      <c r="Q22" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2284,7 +2316,7 @@
         <v>0</v>
       </c>
       <c r="C23" s="3">
-        <f>N23+M23+L23+K23+J23</f>
+        <f t="shared" si="0"/>
         <v>159412.81974307698</v>
       </c>
       <c r="D23">
@@ -2326,8 +2358,11 @@
       <c r="P23">
         <v>0.74298988026741397</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="Q23" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -2335,7 +2370,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="3">
-        <f>N24+M24+L24+K24+J24</f>
+        <f t="shared" si="0"/>
         <v>130424.39365381806</v>
       </c>
       <c r="D24">
@@ -2376,6 +2411,9 @@
       </c>
       <c r="P24">
         <v>0.76093473943346901</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Annual analysis cript updated with equal water production target contraint for all weeks in each month
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2565499F-06C5-4BAA-9BC0-DD86E5B7A389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC3565F-11BF-4838-AF9A-FB0F5E3F0EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
+    <workbookView xWindow="-6375" yWindow="-21600" windowWidth="14175" windowHeight="20985" firstSheet="1" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -294,9 +294,14 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:Q33" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:Q33" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Winter"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="1">
       <filters>
-        <filter val="0"/>
+        <filter val="3"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1204,7 +1209,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1258,7 +1263,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1312,7 +1317,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1366,7 +1371,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1420,7 +1425,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1627,7 +1632,7 @@
         <v>4.8864727960722396</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1681,7 +1686,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1698,7 +1703,7 @@
       <c r="E11">
         <v>10</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="3">
         <v>94059.890410960099</v>
       </c>
       <c r="G11">
@@ -1732,7 +1737,7 @@
         <v>1.7211299327173799</v>
       </c>
     </row>
-    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1749,7 +1754,7 @@
       <c r="E12">
         <v>10</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>117574.86301369801</v>
       </c>
       <c r="G12">
@@ -1783,7 +1788,7 @@
         <v>1.45968753918303</v>
       </c>
     </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1800,7 +1805,7 @@
       <c r="E13">
         <v>10</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="3">
         <v>141089.835616439</v>
       </c>
       <c r="G13">
@@ -1834,7 +1839,7 @@
         <v>1.2818199310829099</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1851,7 +1856,7 @@
       <c r="E14">
         <v>10</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3">
         <v>164604.808219178</v>
       </c>
       <c r="G14">
@@ -1885,7 +1890,7 @@
         <v>1.15734642471583</v>
       </c>
     </row>
-    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1902,7 +1907,7 @@
       <c r="E15">
         <v>10</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="3">
         <v>188119.780821792</v>
       </c>
       <c r="G15">
@@ -1936,7 +1941,7 @@
         <v>1.06438923423513</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1953,7 +1958,7 @@
       <c r="E16">
         <v>10</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>211634.75342465701</v>
       </c>
       <c r="G16">
@@ -1987,7 +1992,7 @@
         <v>0.99711288227329198</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -2041,7 +2046,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2095,7 +2100,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2149,7 +2154,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2203,7 +2208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2257,7 +2262,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2311,7 +2316,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2365,7 +2370,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -2419,7 +2424,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -2473,7 +2478,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -2527,7 +2532,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -2581,7 +2586,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -2635,7 +2640,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -2689,7 +2694,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -2743,7 +2748,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -2797,7 +2802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -2851,7 +2856,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -2907,8 +2912,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>